<commit_message>
Add Cards block variants: Standard, Compact, Feature with colour options
Three card layout variants controlled via CSS classes:
- Standard (default): 3-col grid, image above text, navy colour
- Compact: 2-col, small image floated left beside text, blue colour
- Feature: 2-col, large full-width image above text, blue colour

Colour options: Navy (default) and Blue — applied via .blue class

CSS matches original Tennis NSW site specs:
- White cards with blue box-shadow (#0059CC)
- Absolute-positioned CTA button at bottom (66px height)
- Heading with bottom separator line
- Mobile responsive: single column stacking

Import parser auto-detects variant from source DOM:
- .autoAdjust-3 + .tile--contrast → Standard
- .autoAdjust-2 + .tile--monotone + floated img → Compact
- .autoAdjust-2 + .tile--monotone + block img → Feature

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-section-landing.report.xlsx
+++ b/tools/importer/reports/import-section-landing.report.xlsx
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-01T07:36:36.516Z</t>
+    <t>2026-04-02T06:11:05.694Z</t>
   </si>
   <si>
     <t>Tennis NSW | The governing body of Tennis in New South Wales</t>
@@ -73,7 +73,7 @@
     <t>section-landing</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:59.224Z</t>
+    <t>2026-04-02T07:13:02.390Z</t>
   </si>
   <si>
     <t>About Us | Tennis NSW</t>
@@ -127,7 +127,7 @@
     <t>nsw/players</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:47.511Z</t>
+    <t>2026-04-02T07:12:57.410Z</t>
   </si>
   <si>
     <t>Play | Tennis NSW</t>

</xml_diff>

<commit_message>
Fix card layout: heading above image, variant-specific separators, duplicate banners
Cards JS:
- Extract heading from body and place it BEFORE the image
- Creates .cards-card-heading wrapper above .cards-card-image
- Matches original site order: heading → image → text → CTA

Cards CSS:
- Standard: no separator line under heading
- Compact: 1px solid separator line under heading (blue)
- Feature: no separator line under heading
- Heading styles moved to .cards-card-heading selector

Content fixes:
- Remove duplicate banner images on players, about-us, clubs, our-work
- Apply correct variant classes to clubs (compact blue) and our-work (compact blue)
- Add title blocks to clubs page
- Rebuild section-landing import bundle

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-section-landing.report.xlsx
+++ b/tools/importer/reports/import-section-landing.report.xlsx
@@ -88,7 +88,7 @@
     <t>nsw/clubs</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:43.787Z</t>
+    <t>2026-04-02T07:29:12.200Z</t>
   </si>
   <si>
     <t>Clubs | Tennis NSW</t>
@@ -112,7 +112,7 @@
     <t>nsw/our-work</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:53.285Z</t>
+    <t>2026-04-02T07:29:17.215Z</t>
   </si>
   <si>
     <t>Our Work | Tennis NSW</t>

</xml_diff>